<commit_message>
lear_rabat v9, version endpoints, nginx config, cuadre_asientos, form_generator updates
</commit_message>
<xml_diff>
--- a/standalone_apps/form_generator/excel_storage/registro-visitas.xlsx
+++ b/standalone_apps/form_generator/excel_storage/registro-visitas.xlsx
@@ -426,18 +426,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -448,123 +449,97 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>hora_entrada</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>nombre</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>apellidos</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>dni</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>empresa</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>motivoVisita</t>
-        </is>
-      </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>personaAtiende</t>
+          <t>motivo</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>persona_contacto</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>observaciones</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>aceptaGDPR</t>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>rgpd_consent</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-02-21</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Miguel</t>
+          <t>23:28</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Miguel </t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>del pino</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>75877503c</t>
-        </is>
-      </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>codeengtools</t>
+          <t>75877503C</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Otro</t>
+          <t>Codenegtools</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Jose Luis del Pino</t>
-        </is>
-      </c>
-      <c r="I2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-02-20</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Miguel</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>del Pino</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>75877503C</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Codenegtools</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Entrega</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Jose Luis del Pino</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="b">
+          <t>Reunión</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Jose Luis</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>sdfsdf</t>
+        </is>
+      </c>
+      <c r="J2" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>